<commit_message>
refactor: Simplify local storage functions by removing docstrings and improving readability
</commit_message>
<xml_diff>
--- a/data/requirements.xlsx
+++ b/data/requirements.xlsx
@@ -416,10 +416,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -432,7 +432,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Serial No</t>
+          <t>Lead ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -472,17 +472,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Driver-001</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-22 08:07:02</t>
+          <t>2026-07-07 01:09:37</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>krish Jindal</t>
+          <t>krish</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -492,16 +494,16 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cook</t>
+          <t>Driver</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>delhi</t>
+          <t>dada</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>15000</v>
+        <v>34242</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -510,17 +512,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cook-001</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-22 08:10:47</t>
+          <t>2026-07-07 05:51:57</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>krish Jindal</t>
+          <t xml:space="preserve">krish </t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -530,18 +534,58 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Driver</t>
+          <t>Cook</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>delhi</t>
+          <t>dadad</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>20000</v>
+        <v>133131</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cook-002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-07-07 06:10:17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KRISH JINDAL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8178451022</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cook</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FADA</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>81881</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -558,13 +602,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Serial No</t>
+          <t>Lead ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -644,76 +706,136 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cook-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-07-07 05:51:57</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">krish </t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8178451022</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>krishjindal77@gmail.com</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>dadad</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>dadad</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>dadawd</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>581981</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>133131</v>
+      </c>
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-22 08:07:02</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>krish Jindal</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cook-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-07-07 06:10:17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>KRISH JINDAL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>8178451022</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>krishjindal77@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Rzi-67/68</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>delhi</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>delhi</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>110045</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Afternoon</t>
-        </is>
-      </c>
-      <c r="L2" t="n">
-        <v>15000</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>North Indian</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Should have a friendly nature .</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>KRISHJINDAL@GMAIL.COM</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DADA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FADA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>gc</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>854891</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>81881</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -733,13 +855,13 @@
   <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
@@ -747,14 +869,14 @@
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Serial No</t>
+          <t>Lead ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -834,17 +956,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Driver-001</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-22 08:10:47</t>
+          <t>2026-07-07 01:09:37</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>krish Jindal</t>
+          <t>krish</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -859,27 +983,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>rzi-67/68 mahavir enclave</t>
+          <t>dadad</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>delhi</t>
+          <t>dada</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>delhi</t>
+          <t>dad</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>110045</t>
+          <t>811691</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -888,21 +1012,11 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>20000</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>xuv</t>
-        </is>
+        <v>34242</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>should have a friendly nature</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -928,7 +1042,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Serial No</t>
+          <t>Lead ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">

</xml_diff>

<commit_message>
feat: add PostgreSQL database persistence, modular AI provider support, and tenant authentication services
</commit_message>
<xml_diff>
--- a/data/requirements.xlsx
+++ b/data/requirements.xlsx
@@ -416,17 +416,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,19 +479,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-07 01:09:37</t>
+          <t>2026-09-29 15:48:43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>krish</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
+          <t>Acme Driver Lead</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Driver</t>
@@ -499,11 +495,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dada</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>34242</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -519,19 +515,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-07 05:51:57</t>
+          <t>2026-09-29 15:48:43</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">krish </t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
+          <t>Secret Org B Requirement</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Cook</t>
@@ -539,53 +531,13 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dadad</t>
+          <t>Hyderabad</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>133131</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cook-002</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-07-07 06:10:17</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>KRISH JINDAL</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Cook</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>FADA</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>81881</v>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -602,25 +554,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -713,129 +665,39 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-07 05:51:57</t>
+          <t>2026-09-29 15:48:43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">krish </t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>krishjindal77@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>dadad</t>
-        </is>
-      </c>
+          <t>Secret Org B Requirement</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>dadad</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>dadawd</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>581981</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Morning</t>
-        </is>
-      </c>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>133131</v>
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>South Indian</t>
+        </is>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Cook-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-07-07 06:10:17</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>KRISH JINDAL</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>KRISHJINDAL@GMAIL.COM</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>DADA</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>FADA</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>gc</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>854891</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Morning</t>
-        </is>
-      </c>
-      <c r="L3" t="n">
-        <v>81881</v>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -857,20 +719,20 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -963,62 +825,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-07 01:09:37</t>
+          <t>2026-09-29 15:48:43</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>krish</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>8178451022</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>krishjindal77@gmail.com</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>dadad</t>
-        </is>
-      </c>
+          <t>Acme Driver Lead</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>dada</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>dad</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>811691</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-07-07</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Morning</t>
-        </is>
-      </c>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
-        <v>34242</v>
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>SUV</t>
+        </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>New</t>
@@ -1038,6 +878,24 @@
   </sheetPr>
   <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
feat(ci-cd): implement complete CI/CD architecture with gated Render deployment and health probe verification
</commit_message>
<xml_diff>
--- a/data/requirements.xlsx
+++ b/data/requirements.xlsx
@@ -416,13 +416,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -487,7 +487,6 @@
           <t>Acme Driver Lead</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Driver</t>
@@ -523,7 +522,6 @@
           <t>Secret Org B Requirement</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Cook</t>
@@ -538,6 +536,86 @@
         <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cook-093</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-29 23:21:50</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>API Test Client</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>9820099887</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cook</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cook-099</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:07:10</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>API Test Client</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>9820099887</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cook</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>16000</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -554,14 +632,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -673,18 +751,11 @@
           <t>Secret Org B Requirement</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -696,8 +767,103 @@
       <c r="N2" t="n">
         <v>3</v>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cook-093</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-29 23:21:50</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>API Test Client</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>9820099887</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>apitest@example.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>16000</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>North Indian</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cook-099</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:07:10</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>API Test Client</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>9820099887</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>apitest@example.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>16000</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>North Indian</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>New</t>
         </is>
@@ -833,18 +999,11 @@
           <t>Acme Driver Lead</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Delhi</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -858,7 +1017,6 @@
           <t>Commercial</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>New</t>

</xml_diff>